<commit_message>
Tirage du jour: les 2 exports (jeu + Excel) suivent le toggle ecran Par pays / Chronologique
</commit_message>
<xml_diff>
--- a/TIRAGE_DU_JOUR_28_09_2026_29_tirages_Coloriage_manuel_Miroir_meme_ligne_Miroir_superpose_Memes_numeros_superposes.xlsx
+++ b/TIRAGE_DU_JOUR_28_09_2026_29_tirages_Coloriage_manuel_Miroir_meme_ligne_Miroir_superpose_Memes_numeros_superposes.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAC85351-4E16-544F-A174-ED48A3C0F284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="TIRAGE DU JOUR 28-09-2026 (29 t" state="visible" r:id="rId4"/>
+    <sheet name="TIRAGE DU JOUR 28-09-2026 (29 t" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -235,46 +239,70 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <i/>
+      <sz val="11"/>
       <color rgb="FF6D28D9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF1B5E20"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFBF360C"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF7B5E00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFB71C1C"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF1A1A1A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -382,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -399,6 +427,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -737,41 +766,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P32"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="16" width="8" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="16" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -821,7 +852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -853,7 +884,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -903,7 +934,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -953,7 +984,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4</v>
       </c>
@@ -1003,7 +1034,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -1053,7 +1084,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6</v>
       </c>
@@ -1103,7 +1134,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -1153,7 +1184,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -1203,7 +1234,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -1253,7 +1284,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>10</v>
       </c>
@@ -1303,7 +1334,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>11</v>
       </c>
@@ -1335,7 +1366,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>12</v>
       </c>
@@ -1385,7 +1416,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>13</v>
       </c>
@@ -1417,7 +1448,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>14</v>
       </c>
@@ -1467,7 +1498,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>15</v>
       </c>
@@ -1517,7 +1548,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>16</v>
       </c>
@@ -1567,7 +1598,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>17</v>
       </c>
@@ -1617,7 +1648,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>18</v>
       </c>
@@ -1667,7 +1698,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>19</v>
       </c>
@@ -1717,7 +1748,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>20</v>
       </c>
@@ -1767,7 +1798,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>21</v>
       </c>
@@ -1799,7 +1830,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>22</v>
       </c>
@@ -1849,7 +1880,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>23</v>
       </c>
@@ -1881,7 +1912,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>24</v>
       </c>
@@ -1913,7 +1944,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>25</v>
       </c>
@@ -1945,7 +1976,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>26</v>
       </c>
@@ -1977,7 +2008,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>27</v>
       </c>
@@ -2027,7 +2058,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>28</v>
       </c>
@@ -2059,7 +2090,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>29</v>
       </c>
@@ -2096,6 +2127,6 @@
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>